<commit_message>
update acceptance testing and project report
</commit_message>
<xml_diff>
--- a/Project/Documentation/Test-Cases.xlsx
+++ b/Project/Documentation/Test-Cases.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\bolfa\VIA\BPR1\Project\Documentation\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0753F33-85A4-4D6E-9DEB-85281F5DD8B2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C48E44D8-B312-4E4E-B41C-9C3CF2DED6CE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="825" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21120" tabRatio="825" firstSheet="2" activeTab="5" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Register an account" sheetId="7" r:id="rId1"/>
@@ -18,11 +18,12 @@
     <sheet name="Log in" sheetId="6" r:id="rId3"/>
     <sheet name="Reset password" sheetId="10" r:id="rId4"/>
     <sheet name="Log out" sheetId="20" r:id="rId5"/>
-    <sheet name="Link account" sheetId="12" r:id="rId6"/>
-    <sheet name="Manage provider connection" sheetId="14" r:id="rId7"/>
+    <sheet name="Link provider's account" sheetId="12" r:id="rId6"/>
+    <sheet name="Manage provider's connection" sheetId="14" r:id="rId7"/>
     <sheet name="Browse unified files" sheetId="16" r:id="rId8"/>
     <sheet name="Cross-provider search" sheetId="17" r:id="rId9"/>
-    <sheet name="Open item &amp; see metadata" sheetId="18" r:id="rId10"/>
+    <sheet name="See item's metadata" sheetId="18" r:id="rId10"/>
+    <sheet name="Open item in provider" sheetId="21" r:id="rId11"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -45,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="204">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="426" uniqueCount="202">
   <si>
     <t xml:space="preserve">Test scenarios for case A </t>
   </si>
@@ -314,9 +315,6 @@
     <t>Token stored (access + refresh)</t>
   </si>
   <si>
-    <t>State  = Connected</t>
-  </si>
-  <si>
     <t>Denies consent</t>
   </si>
   <si>
@@ -332,39 +330,24 @@
     <t>Consent = Allow</t>
   </si>
   <si>
-    <t>Code = Valid</t>
-  </si>
-  <si>
-    <t>Expected: Tokens saved (encrypted), status Connected</t>
-  </si>
-  <si>
     <t>TC2 - Deny</t>
   </si>
   <si>
     <t>Consent = Deny</t>
   </si>
   <si>
-    <t>Expected: Back to app with "Not connected"</t>
-  </si>
-  <si>
     <t>TC3 - Invalid code</t>
   </si>
   <si>
     <t>Code = empty/invalid</t>
   </si>
   <si>
-    <t>Expected: "Reconnect" prompt, no token stored</t>
-  </si>
-  <si>
     <t>TC4 - Exchange fails</t>
   </si>
   <si>
     <t>Provider 500 during token exchange</t>
   </si>
   <si>
-    <t>Expected: Error shown, status Not connected</t>
-  </si>
-  <si>
     <t>Active session</t>
   </si>
   <si>
@@ -596,21 +579,6 @@
     <t>Permission denied/not found</t>
   </si>
   <si>
-    <t>B: Metadata</t>
-  </si>
-  <si>
-    <t>Show metadata panel for selected item</t>
-  </si>
-  <si>
-    <t>Item selected/valid item ID</t>
-  </si>
-  <si>
-    <t>Item not selecteds/invalid item ID</t>
-  </si>
-  <si>
-    <t>Show no metadata panel</t>
-  </si>
-  <si>
     <t>TC1 - Open OK</t>
   </si>
   <si>
@@ -647,16 +615,43 @@
     <t>Expected: Error, stay in app</t>
   </si>
   <si>
-    <t>TC5 - Show metadata</t>
-  </si>
-  <si>
-    <t>Expected: Fields populated (name, size, modified, provider)</t>
-  </si>
-  <si>
-    <t>TC5 - Metadata with invalid item</t>
-  </si>
-  <si>
-    <t>Expected: Error state, panel closed</t>
+    <t>A: Metadata</t>
+  </si>
+  <si>
+    <t>User selects an item to view metadata</t>
+  </si>
+  <si>
+    <t>System shows the item's metadata (name, size, modified, provider)</t>
+  </si>
+  <si>
+    <t>ALT</t>
+  </si>
+  <si>
+    <t>Invalid or unselected item ID</t>
+  </si>
+  <si>
+    <t>System shows no metadata (or error state)</t>
+  </si>
+  <si>
+    <t>State = Connected</t>
+  </si>
+  <si>
+    <t>Callback Code = Valid</t>
+  </si>
+  <si>
+    <t>Actualt result: Same</t>
+  </si>
+  <si>
+    <t>Expected result: Tokens saved (encrypted), status Connected</t>
+  </si>
+  <si>
+    <t>Expected result: Back to app with "Not connected"</t>
+  </si>
+  <si>
+    <t>Expected result: "Reconnect" prompt, no token stored</t>
+  </si>
+  <si>
+    <t>Expected result: Error shown, status Not connected</t>
   </si>
 </sst>
 </file>
@@ -791,7 +786,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="15">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -971,11 +966,37 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="105">
+  <cellXfs count="126">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -1037,9 +1058,6 @@
     <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="11" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
@@ -1068,9 +1086,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="14" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1120,9 +1135,6 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="11" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
@@ -1212,11 +1224,14 @@
     <xf numFmtId="0" fontId="0" fillId="11" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="15" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="14" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="16" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1233,31 +1248,16 @@
     <xf numFmtId="0" fontId="4" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="13" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="15" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="12" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1269,11 +1269,95 @@
     <xf numFmtId="0" fontId="0" fillId="7" borderId="14" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="14" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="9" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="7" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="9" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="11" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="11" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="14" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="15" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1521,21 +1605,21 @@
       <c r="M1" s="12"/>
     </row>
     <row r="2" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="54" t="s">
         <v>34</v>
       </c>
-      <c r="B2" s="57"/>
-      <c r="C2" s="57"/>
-      <c r="D2" s="57"/>
-      <c r="E2" s="57"/>
+      <c r="B2" s="54"/>
+      <c r="C2" s="54"/>
+      <c r="D2" s="54"/>
+      <c r="E2" s="54"/>
       <c r="F2" s="14"/>
-      <c r="G2" s="57" t="s">
+      <c r="G2" s="54" t="s">
         <v>1</v>
       </c>
-      <c r="H2" s="57"/>
-      <c r="I2" s="57"/>
-      <c r="J2" s="57"/>
-      <c r="K2" s="57"/>
+      <c r="H2" s="54"/>
+      <c r="I2" s="54"/>
+      <c r="J2" s="54"/>
+      <c r="K2" s="54"/>
       <c r="O2" s="12"/>
       <c r="P2" s="12"/>
       <c r="Q2" s="12"/>
@@ -1687,7 +1771,7 @@
       <c r="S8" s="12"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A9" s="58" t="s">
+      <c r="A9" s="55" t="s">
         <v>14</v>
       </c>
       <c r="B9" s="16" t="s">
@@ -1699,16 +1783,16 @@
       <c r="D9" s="16" t="s">
         <v>23</v>
       </c>
-      <c r="G9" s="57" t="s">
+      <c r="G9" s="54" t="s">
         <v>20</v>
       </c>
-      <c r="H9" s="57"/>
-      <c r="I9" s="57"/>
-      <c r="J9" s="57"/>
-      <c r="K9" s="57"/>
+      <c r="H9" s="54"/>
+      <c r="I9" s="54"/>
+      <c r="J9" s="54"/>
+      <c r="K9" s="54"/>
     </row>
     <row r="10" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="59"/>
+      <c r="A10" s="56"/>
       <c r="B10" s="16" t="s">
         <v>17</v>
       </c>
@@ -1753,7 +1837,7 @@
       </c>
     </row>
     <row r="12" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A12" s="60" t="s">
+      <c r="A12" s="57" t="s">
         <v>35</v>
       </c>
       <c r="B12" s="18" t="s">
@@ -1778,18 +1862,18 @@
       </c>
     </row>
     <row r="13" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="61"/>
+      <c r="A13" s="58"/>
       <c r="B13" s="18" t="s">
         <v>17</v>
       </c>
       <c r="C13" s="18" t="s">
         <v>18</v>
       </c>
-      <c r="O13" s="55"/>
-      <c r="P13" s="56"/>
-      <c r="Q13" s="56"/>
-      <c r="R13" s="56"/>
-      <c r="S13" s="56"/>
+      <c r="O13" s="52"/>
+      <c r="P13" s="53"/>
+      <c r="Q13" s="53"/>
+      <c r="R13" s="53"/>
+      <c r="S13" s="53"/>
     </row>
     <row r="14" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="O14" s="12"/>
@@ -1806,13 +1890,13 @@
       <c r="S15" s="12"/>
     </row>
     <row r="16" spans="1:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G16" s="57" t="s">
+      <c r="G16" s="54" t="s">
         <v>24</v>
       </c>
-      <c r="H16" s="57"/>
-      <c r="I16" s="57"/>
-      <c r="J16" s="57"/>
-      <c r="K16" s="57"/>
+      <c r="H16" s="54"/>
+      <c r="I16" s="54"/>
+      <c r="J16" s="54"/>
+      <c r="K16" s="54"/>
       <c r="O16" s="12"/>
       <c r="P16" s="12"/>
       <c r="Q16" s="12"/>
@@ -1889,13 +1973,13 @@
     <row r="21" spans="7:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="22" spans="7:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2"/>
     <row r="23" spans="7:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="G23" s="57" t="s">
+      <c r="G23" s="54" t="s">
         <v>2</v>
       </c>
-      <c r="H23" s="57"/>
-      <c r="I23" s="57"/>
-      <c r="J23" s="57"/>
-      <c r="K23" s="57"/>
+      <c r="H23" s="54"/>
+      <c r="I23" s="54"/>
+      <c r="J23" s="54"/>
+      <c r="K23" s="54"/>
     </row>
     <row r="24" spans="7:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="G24" s="15" t="s">
@@ -1913,11 +1997,11 @@
       <c r="K24" s="15" t="s">
         <v>13</v>
       </c>
-      <c r="N24" s="55"/>
-      <c r="O24" s="56"/>
-      <c r="P24" s="56"/>
-      <c r="Q24" s="56"/>
-      <c r="R24" s="56"/>
+      <c r="N24" s="52"/>
+      <c r="O24" s="53"/>
+      <c r="P24" s="53"/>
+      <c r="Q24" s="53"/>
+      <c r="R24" s="53"/>
     </row>
     <row r="25" spans="7:19" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="G25" s="16" t="s">
@@ -3096,234 +3180,386 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BA487E22-3AE1-4F27-B490-76D7F721B5ED}">
+  <dimension ref="A1:D30"/>
+  <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="1" width="17.85546875" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="39.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="61.42578125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A1" s="93" t="s">
+        <v>41</v>
+      </c>
+      <c r="B1" s="94"/>
+      <c r="C1" s="95"/>
+      <c r="D1" s="19"/>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A2" s="43" t="s">
+        <v>189</v>
+      </c>
+      <c r="B2" s="46" t="s">
+        <v>190</v>
+      </c>
+      <c r="C2" s="43" t="s">
+        <v>191</v>
+      </c>
+      <c r="D2" s="48"/>
+    </row>
+    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A3" s="42" t="s">
+        <v>192</v>
+      </c>
+      <c r="B3" s="42" t="s">
+        <v>193</v>
+      </c>
+      <c r="C3" s="42" t="s">
+        <v>194</v>
+      </c>
+      <c r="D3" s="13"/>
+    </row>
+    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A4" s="101"/>
+      <c r="B4" s="104"/>
+      <c r="C4" s="100"/>
+      <c r="D4" s="13"/>
+    </row>
+    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A5" s="102"/>
+      <c r="B5" s="102"/>
+      <c r="C5" s="102"/>
+      <c r="D5" s="13"/>
+    </row>
+    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A6" s="102"/>
+      <c r="B6" s="102"/>
+      <c r="C6" s="102"/>
+      <c r="D6" s="13"/>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A7" s="103"/>
+      <c r="B7" s="103"/>
+      <c r="C7" s="103"/>
+      <c r="D7" s="13"/>
+    </row>
+    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A8" s="19"/>
+      <c r="B8" s="19"/>
+      <c r="C8" s="19"/>
+      <c r="D8" s="50"/>
+    </row>
+    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A9" s="19"/>
+      <c r="B9" s="19"/>
+      <c r="C9" s="19"/>
+      <c r="D9" s="48"/>
+    </row>
+    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A10" s="19"/>
+      <c r="B10" s="19"/>
+      <c r="C10" s="19"/>
+      <c r="D10" s="13"/>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A11" s="19"/>
+      <c r="B11" s="19"/>
+      <c r="C11" s="19"/>
+      <c r="D11" s="50"/>
+    </row>
+    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A12" s="19"/>
+      <c r="B12" s="19"/>
+      <c r="C12" s="19"/>
+      <c r="D12" s="48"/>
+    </row>
+    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A13" s="19"/>
+      <c r="B13" s="19"/>
+      <c r="C13" s="19"/>
+      <c r="D13" s="13"/>
+    </row>
+    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A14" s="19"/>
+      <c r="B14" s="19"/>
+      <c r="C14" s="19"/>
+      <c r="D14" s="50"/>
+    </row>
+    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A15" s="19"/>
+      <c r="B15" s="19"/>
+      <c r="C15" s="19"/>
+      <c r="D15" s="48"/>
+    </row>
+    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A16" s="19"/>
+      <c r="B16" s="19"/>
+      <c r="C16" s="19"/>
+      <c r="D16" s="13"/>
+    </row>
+    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A17" s="19"/>
+      <c r="B17" s="19"/>
+      <c r="C17" s="19"/>
+      <c r="D17" s="50"/>
+    </row>
+    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A18" s="19"/>
+      <c r="B18" s="19"/>
+      <c r="C18" s="19"/>
+      <c r="D18" s="50"/>
+    </row>
+    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A19" s="19"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="23"/>
+    </row>
+    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A20" s="19"/>
+      <c r="B20" s="19"/>
+      <c r="C20" s="19"/>
+      <c r="D20" s="50"/>
+    </row>
+    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A21" s="19"/>
+      <c r="B21" s="19"/>
+      <c r="C21" s="19"/>
+      <c r="D21" s="48"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="19"/>
+      <c r="B22" s="19"/>
+      <c r="C22" s="19"/>
+    </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A23" s="19"/>
+      <c r="B23" s="19"/>
+      <c r="C23" s="19"/>
+    </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A24" s="19"/>
+      <c r="B24" s="19"/>
+      <c r="C24" s="19"/>
+    </row>
+    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A25" s="19"/>
+      <c r="B25" s="19"/>
+      <c r="C25" s="19"/>
+    </row>
+    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A26" s="19"/>
+      <c r="B26" s="19"/>
+      <c r="C26" s="19"/>
+    </row>
+    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A27" s="19"/>
+      <c r="B27" s="19"/>
+      <c r="C27" s="19"/>
+    </row>
+    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A28" s="19"/>
+      <c r="B28" s="19"/>
+      <c r="C28" s="19"/>
+    </row>
+    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A29" s="19"/>
+      <c r="B29" s="19"/>
+      <c r="C29" s="19"/>
+    </row>
+    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A30" s="19"/>
+      <c r="B30" s="19"/>
+      <c r="C30" s="19"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A1:C1"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{5BFB6702-C84A-451D-A5F7-9836C552A77F}">
   <dimension ref="A1:D24"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="16.85546875" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="28.85546875" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="51.28515625" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="15.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="100" t="s">
+    <row r="1" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A1" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="102"/>
-      <c r="D1" s="19"/>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="45" t="s">
+      <c r="B1" s="94"/>
+      <c r="C1" s="95"/>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A2" s="43" t="s">
+        <v>173</v>
+      </c>
+      <c r="B2" s="46" t="s">
+        <v>174</v>
+      </c>
+      <c r="C2" s="43"/>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A3" s="42" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="47" t="s">
+        <v>49</v>
+      </c>
+      <c r="C3" s="42" t="s">
+        <v>175</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A4" s="41" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="51" t="s">
+        <v>176</v>
+      </c>
+      <c r="C4" s="22"/>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A5" s="101"/>
+      <c r="B5" s="101"/>
+      <c r="C5" s="101"/>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A6" s="105" t="s">
+        <v>177</v>
+      </c>
+      <c r="B6" s="106"/>
+      <c r="C6" s="107"/>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A7" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B7" s="40" t="s">
+        <v>178</v>
+      </c>
+      <c r="C7" s="40" t="s">
         <v>179</v>
       </c>
-      <c r="B2" s="48" t="s">
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A8" s="13"/>
+      <c r="B8" s="13"/>
+      <c r="C8" s="13"/>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A9" s="34" t="s">
         <v>180</v>
       </c>
-      <c r="C2" s="45"/>
-      <c r="D2" s="51"/>
-    </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="44" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="49" t="s">
-        <v>49</v>
-      </c>
-      <c r="C3" s="44" t="s">
+      <c r="B9" s="34"/>
+      <c r="C9" s="34"/>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A10" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B10" s="40" t="s">
         <v>181</v>
       </c>
-      <c r="D3" s="13"/>
-    </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A4" s="43" t="s">
-        <v>58</v>
-      </c>
-      <c r="B4" s="54" t="s">
+      <c r="C10" s="40" t="s">
         <v>182</v>
       </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="13"/>
-    </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="39" t="s">
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A11" s="13"/>
+      <c r="B11" s="13"/>
+      <c r="C11" s="13"/>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A12" s="34" t="s">
         <v>183</v>
       </c>
-      <c r="B5" s="50" t="s">
+      <c r="B12" s="34"/>
+      <c r="C12" s="34"/>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A13" s="29" t="s">
+        <v>66</v>
+      </c>
+      <c r="B13" s="45" t="s">
+        <v>184</v>
+      </c>
+      <c r="C13" s="40" t="s">
         <v>185</v>
       </c>
-      <c r="C5" s="39" t="s">
-        <v>184</v>
-      </c>
-      <c r="D5" s="13"/>
-    </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="39"/>
-      <c r="B6" s="50" t="s">
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A14" s="13"/>
+      <c r="B14" s="13"/>
+      <c r="C14" s="13"/>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A15" s="90" t="s">
         <v>186</v>
       </c>
-      <c r="C6" s="39" t="s">
+      <c r="B15" s="90"/>
+      <c r="C15" s="90"/>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.2">
+      <c r="A16" s="27" t="s">
+        <v>66</v>
+      </c>
+      <c r="B16" s="45" t="s">
         <v>187</v>
       </c>
-      <c r="D6" s="13"/>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A7" s="13"/>
-      <c r="B7" s="13"/>
-      <c r="C7" s="13"/>
-      <c r="D7" s="13"/>
-    </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="98" t="s">
+      <c r="C16" s="33" t="s">
         <v>188</v>
       </c>
-      <c r="B8" s="98"/>
-      <c r="C8" s="98"/>
-      <c r="D8" s="53"/>
-    </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="B9" s="42" t="s">
-        <v>189</v>
-      </c>
-      <c r="C9" s="42" t="s">
-        <v>190</v>
-      </c>
-      <c r="D9" s="51"/>
-    </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A10" s="13"/>
-      <c r="B10" s="13"/>
-      <c r="C10" s="13"/>
-      <c r="D10" s="13"/>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A11" s="99" t="s">
-        <v>191</v>
-      </c>
-      <c r="B11" s="99"/>
-      <c r="C11" s="99"/>
-      <c r="D11" s="53"/>
-    </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="B12" s="42" t="s">
-        <v>192</v>
-      </c>
-      <c r="C12" s="42" t="s">
-        <v>193</v>
-      </c>
-      <c r="D12" s="51"/>
-    </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="13"/>
-      <c r="B13" s="13"/>
-      <c r="C13" s="13"/>
-      <c r="D13" s="13"/>
-    </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A14" s="99" t="s">
-        <v>194</v>
-      </c>
-      <c r="B14" s="99"/>
-      <c r="C14" s="99"/>
-      <c r="D14" s="53"/>
-    </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="B15" s="47" t="s">
-        <v>195</v>
-      </c>
-      <c r="C15" s="42" t="s">
-        <v>196</v>
-      </c>
-      <c r="D15" s="51"/>
-    </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="13"/>
-      <c r="B16" s="13"/>
-      <c r="C16" s="13"/>
-      <c r="D16" s="13"/>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A17" s="94" t="s">
-        <v>197</v>
-      </c>
-      <c r="B17" s="94"/>
-      <c r="C17" s="94"/>
-      <c r="D17" s="53"/>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A18" s="28" t="s">
-        <v>66</v>
-      </c>
-      <c r="B18" s="47" t="s">
-        <v>198</v>
-      </c>
-      <c r="C18" s="35" t="s">
-        <v>199</v>
-      </c>
-      <c r="D18" s="53"/>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A19" s="24"/>
-      <c r="B19" s="24"/>
-      <c r="C19" s="24"/>
-      <c r="D19" s="24"/>
+      <c r="A19" s="23"/>
+      <c r="B19" s="23"/>
+      <c r="C19" s="23"/>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A20" s="95" t="s">
-        <v>200</v>
-      </c>
-      <c r="B20" s="95"/>
-      <c r="C20" s="95"/>
-      <c r="D20" s="53"/>
+      <c r="A20" s="102"/>
+      <c r="B20" s="102"/>
+      <c r="C20" s="102"/>
+      <c r="D20" s="102"/>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A21" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="B21" s="42" t="s">
-        <v>185</v>
-      </c>
-      <c r="C21" s="42" t="s">
-        <v>201</v>
-      </c>
-      <c r="D21" s="51"/>
+      <c r="A21" s="102"/>
+      <c r="B21" s="102"/>
+      <c r="C21" s="102"/>
+      <c r="D21" s="102"/>
+    </row>
+    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A22" s="102"/>
+      <c r="B22" s="102"/>
+      <c r="C22" s="102"/>
+      <c r="D22" s="102"/>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A23" s="95" t="s">
-        <v>202</v>
-      </c>
-      <c r="B23" s="95"/>
-      <c r="C23" s="95"/>
+      <c r="A23" s="102"/>
+      <c r="B23" s="102"/>
+      <c r="C23" s="102"/>
+      <c r="D23" s="102"/>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A24" s="30" t="s">
-        <v>66</v>
-      </c>
-      <c r="B24" s="42" t="s">
-        <v>186</v>
-      </c>
-      <c r="C24" s="47" t="s">
-        <v>203</v>
-      </c>
+      <c r="A24" s="102"/>
+      <c r="B24" s="102"/>
+      <c r="C24" s="102"/>
+      <c r="D24" s="102"/>
     </row>
   </sheetData>
-  <mergeCells count="7">
+  <mergeCells count="3">
+    <mergeCell ref="A6:C6"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A23:C23"/>
-    <mergeCell ref="A20:C20"/>
-    <mergeCell ref="A17:C17"/>
-    <mergeCell ref="A14:C14"/>
-    <mergeCell ref="A11:C11"/>
-    <mergeCell ref="A8:C8"/>
+    <mergeCell ref="A15:C15"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -3342,11 +3578,11 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="61" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" s="20" t="s">
@@ -3360,101 +3596,101 @@
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="B3" s="21" t="s">
         <v>84</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C3" s="21" t="s">
         <v>85</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="62" t="s">
+      <c r="A5" s="59" t="s">
         <v>60</v>
       </c>
-      <c r="B5" s="62"/>
-      <c r="C5" s="62"/>
-      <c r="D5" s="62"/>
+      <c r="B5" s="59"/>
+      <c r="C5" s="59"/>
+      <c r="D5" s="59"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="30" t="s">
+      <c r="A6" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="30" t="s">
+      <c r="B6" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="30" t="s">
+      <c r="C6" s="29" t="s">
         <v>47</v>
       </c>
-      <c r="D6" s="30" t="s">
+      <c r="D6" s="29" t="s">
         <v>50</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="63" t="s">
+      <c r="A8" s="60" t="s">
         <v>48</v>
       </c>
-      <c r="B8" s="63"/>
-      <c r="C8" s="63"/>
-      <c r="D8" s="63"/>
+      <c r="B8" s="60"/>
+      <c r="C8" s="60"/>
+      <c r="D8" s="60"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="30" t="s">
+      <c r="A9" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B9" s="30" t="s">
+      <c r="B9" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="C9" s="30" t="s">
+      <c r="C9" s="29" t="s">
         <v>49</v>
       </c>
-      <c r="D9" s="30" t="s">
+      <c r="D9" s="29" t="s">
         <v>51</v>
       </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A12" s="63" t="s">
+      <c r="A12" s="60" t="s">
         <v>52</v>
       </c>
-      <c r="B12" s="63"/>
-      <c r="C12" s="63"/>
-      <c r="D12" s="63"/>
+      <c r="B12" s="60"/>
+      <c r="C12" s="60"/>
+      <c r="D12" s="60"/>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A13" s="30" t="s">
+      <c r="A13" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B13" s="30" t="s">
+      <c r="B13" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="C13" s="30" t="s">
+      <c r="C13" s="29" t="s">
         <v>53</v>
       </c>
-      <c r="D13" s="30" t="s">
+      <c r="D13" s="29" t="s">
         <v>54</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A15" s="63" t="s">
+      <c r="A15" s="60" t="s">
         <v>55</v>
       </c>
-      <c r="B15" s="63"/>
-      <c r="C15" s="63"/>
-      <c r="D15" s="63"/>
+      <c r="B15" s="60"/>
+      <c r="C15" s="60"/>
+      <c r="D15" s="60"/>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A16" s="30" t="s">
+      <c r="A16" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B16" s="30" t="s">
+      <c r="B16" s="29" t="s">
         <v>46</v>
       </c>
-      <c r="C16" s="30" t="s">
+      <c r="C16" s="29" t="s">
         <v>56</v>
       </c>
-      <c r="D16" s="30" t="s">
+      <c r="D16" s="29" t="s">
         <v>57</v>
       </c>
     </row>
@@ -3526,39 +3762,39 @@
       <c r="Z1" s="8"/>
     </row>
     <row r="2" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A2" s="70" t="s">
+      <c r="A2" s="67" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="71"/>
-      <c r="C2" s="71"/>
-      <c r="D2" s="71"/>
-      <c r="E2" s="71"/>
-      <c r="F2" s="71"/>
-      <c r="G2" s="72"/>
+      <c r="B2" s="68"/>
+      <c r="C2" s="68"/>
+      <c r="D2" s="68"/>
+      <c r="E2" s="68"/>
+      <c r="F2" s="68"/>
+      <c r="G2" s="69"/>
       <c r="H2" s="1"/>
-      <c r="I2" s="67" t="s">
+      <c r="I2" s="64" t="s">
         <v>1</v>
       </c>
-      <c r="J2" s="68"/>
-      <c r="K2" s="68"/>
-      <c r="L2" s="68"/>
-      <c r="M2" s="69"/>
+      <c r="J2" s="65"/>
+      <c r="K2" s="65"/>
+      <c r="L2" s="65"/>
+      <c r="M2" s="66"/>
       <c r="N2" s="1"/>
-      <c r="O2" s="67" t="s">
+      <c r="O2" s="64" t="s">
         <v>20</v>
       </c>
-      <c r="P2" s="68"/>
-      <c r="Q2" s="68"/>
-      <c r="R2" s="68"/>
-      <c r="S2" s="69"/>
+      <c r="P2" s="65"/>
+      <c r="Q2" s="65"/>
+      <c r="R2" s="65"/>
+      <c r="S2" s="66"/>
       <c r="T2" s="8"/>
-      <c r="U2" s="67" t="s">
+      <c r="U2" s="64" t="s">
         <v>24</v>
       </c>
-      <c r="V2" s="68"/>
-      <c r="W2" s="68"/>
-      <c r="X2" s="68"/>
-      <c r="Y2" s="69"/>
+      <c r="V2" s="65"/>
+      <c r="W2" s="65"/>
+      <c r="X2" s="65"/>
+      <c r="Y2" s="66"/>
       <c r="Z2" s="8"/>
     </row>
     <row r="3" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
@@ -3794,7 +4030,7 @@
       <c r="Z6" s="8"/>
     </row>
     <row r="7" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="73" t="s">
+      <c r="A7" s="70" t="s">
         <v>14</v>
       </c>
       <c r="B7" s="10" t="s">
@@ -3809,33 +4045,33 @@
       <c r="F7" s="1"/>
       <c r="G7" s="1"/>
       <c r="H7" s="1"/>
-      <c r="I7" s="67" t="s">
+      <c r="I7" s="64" t="s">
         <v>2</v>
       </c>
-      <c r="J7" s="68"/>
-      <c r="K7" s="68"/>
-      <c r="L7" s="68"/>
-      <c r="M7" s="69"/>
+      <c r="J7" s="65"/>
+      <c r="K7" s="65"/>
+      <c r="L7" s="65"/>
+      <c r="M7" s="66"/>
       <c r="N7" s="1"/>
-      <c r="O7" s="67" t="s">
+      <c r="O7" s="64" t="s">
         <v>21</v>
       </c>
-      <c r="P7" s="68"/>
-      <c r="Q7" s="68"/>
-      <c r="R7" s="68"/>
-      <c r="S7" s="69"/>
+      <c r="P7" s="65"/>
+      <c r="Q7" s="65"/>
+      <c r="R7" s="65"/>
+      <c r="S7" s="66"/>
       <c r="T7" s="1"/>
-      <c r="U7" s="67" t="s">
+      <c r="U7" s="64" t="s">
         <v>25</v>
       </c>
-      <c r="V7" s="68"/>
-      <c r="W7" s="68"/>
-      <c r="X7" s="68"/>
-      <c r="Y7" s="69"/>
+      <c r="V7" s="65"/>
+      <c r="W7" s="65"/>
+      <c r="X7" s="65"/>
+      <c r="Y7" s="66"/>
       <c r="Z7" s="8"/>
     </row>
     <row r="8" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="66"/>
+      <c r="A8" s="63"/>
       <c r="B8" s="10" t="s">
         <v>17</v>
       </c>
@@ -3954,7 +4190,7 @@
       <c r="Z9" s="8"/>
     </row>
     <row r="10" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="65" t="s">
+      <c r="A10" s="62" t="s">
         <v>16</v>
       </c>
       <c r="B10" s="11" t="s">
@@ -4013,7 +4249,7 @@
       <c r="Z10" s="8"/>
     </row>
     <row r="11" spans="1:26" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="66"/>
+      <c r="A11" s="63"/>
       <c r="B11" s="11" t="s">
         <v>17</v>
       </c>
@@ -10631,28 +10867,28 @@
   <dimension ref="A1:K64"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7" style="24" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="55.42578125" style="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="43.42578125" style="24" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="23" style="24" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="8" style="24" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="3.7109375" style="24" customWidth="1"/>
-    <col min="7" max="7" width="21" style="24" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9.5703125" style="24" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="15" style="24" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="14.85546875" style="24" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="12.140625" style="24" bestFit="1" customWidth="1"/>
-    <col min="12" max="16384" width="9.140625" style="24"/>
+    <col min="1" max="1" width="7" style="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="55.42578125" style="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="43.42578125" style="23" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="23" style="23" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="8" style="23" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="3.7109375" style="23" customWidth="1"/>
+    <col min="7" max="7" width="21" style="23" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="9.5703125" style="23" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="15" style="23" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="14.85546875" style="23" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12.140625" style="23" bestFit="1" customWidth="1"/>
+    <col min="12" max="16384" width="9.140625" style="23"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A1" s="64" t="s">
+      <c r="A1" s="61" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="64"/>
-      <c r="C1" s="64"/>
-      <c r="D1" s="64"/>
-      <c r="E1" s="64"/>
+      <c r="B1" s="61"/>
+      <c r="C1" s="61"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="61"/>
       <c r="F1" s="13"/>
       <c r="G1" s="13"/>
       <c r="H1" s="13"/>
@@ -10673,7 +10909,7 @@
       <c r="D2" s="20" t="s">
         <v>79</v>
       </c>
-      <c r="E2" s="25" t="s">
+      <c r="E2" s="24" t="s">
         <v>80</v>
       </c>
       <c r="F2" s="14"/>
@@ -10684,15 +10920,15 @@
       <c r="K2" s="12"/>
     </row>
     <row r="3" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
         <v>45</v>
       </c>
-      <c r="B3" s="63" t="s">
+      <c r="B3" s="60" t="s">
         <v>81</v>
       </c>
-      <c r="C3" s="63"/>
-      <c r="D3" s="63"/>
-      <c r="E3" s="63"/>
+      <c r="C3" s="60"/>
+      <c r="D3" s="60"/>
+      <c r="E3" s="60"/>
       <c r="F3" s="12"/>
       <c r="G3" s="12"/>
       <c r="H3" s="12"/>
@@ -10701,15 +10937,15 @@
       <c r="K3" s="12"/>
     </row>
     <row r="4" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A4" s="23" t="s">
+      <c r="A4" s="22" t="s">
         <v>58</v>
       </c>
-      <c r="B4" s="74" t="s">
+      <c r="B4" s="71" t="s">
         <v>82</v>
       </c>
-      <c r="C4" s="74"/>
-      <c r="D4" s="74"/>
-      <c r="E4" s="74"/>
+      <c r="C4" s="71"/>
+      <c r="D4" s="71"/>
+      <c r="E4" s="71"/>
       <c r="F4" s="12"/>
       <c r="G4" s="12"/>
       <c r="H4" s="12"/>
@@ -10731,11 +10967,11 @@
       <c r="K5" s="12"/>
     </row>
     <row r="6" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A6" s="62" t="s">
+      <c r="A6" s="59" t="s">
         <v>59</v>
       </c>
-      <c r="B6" s="62"/>
-      <c r="C6" s="62"/>
+      <c r="B6" s="59"/>
+      <c r="C6" s="59"/>
       <c r="D6" s="13"/>
       <c r="E6" s="13"/>
       <c r="F6" s="13"/>
@@ -10746,13 +10982,13 @@
       <c r="K6" s="13"/>
     </row>
     <row r="7" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A7" s="30" t="s">
+      <c r="A7" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B7" s="30" t="s">
+      <c r="B7" s="29" t="s">
         <v>64</v>
       </c>
-      <c r="C7" s="30" t="s">
+      <c r="C7" s="29" t="s">
         <v>65</v>
       </c>
       <c r="D7" s="13"/>
@@ -10765,13 +11001,13 @@
       <c r="K7" s="13"/>
     </row>
     <row r="8" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A8" s="30" t="s">
+      <c r="A8" s="29" t="s">
         <v>67</v>
       </c>
-      <c r="B8" s="30" t="s">
+      <c r="B8" s="29" t="s">
         <v>68</v>
       </c>
-      <c r="C8" s="30" t="s">
+      <c r="C8" s="29" t="s">
         <v>69</v>
       </c>
       <c r="D8" s="13"/>
@@ -10797,11 +11033,11 @@
       <c r="K9" s="12"/>
     </row>
     <row r="10" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A10" s="63" t="s">
+      <c r="A10" s="60" t="s">
         <v>61</v>
       </c>
-      <c r="B10" s="63"/>
-      <c r="C10" s="63"/>
+      <c r="B10" s="60"/>
+      <c r="C10" s="60"/>
       <c r="D10" s="13"/>
       <c r="E10" s="13"/>
       <c r="F10" s="13"/>
@@ -10812,13 +11048,13 @@
       <c r="K10" s="12"/>
     </row>
     <row r="11" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B11" s="30" t="s">
+      <c r="B11" s="29" t="s">
         <v>70</v>
       </c>
-      <c r="C11" s="30" t="s">
+      <c r="C11" s="29" t="s">
         <v>71</v>
       </c>
       <c r="D11" s="13"/>
@@ -10844,11 +11080,11 @@
       <c r="K12" s="12"/>
     </row>
     <row r="13" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A13" s="74" t="s">
+      <c r="A13" s="71" t="s">
         <v>62</v>
       </c>
-      <c r="B13" s="74"/>
-      <c r="C13" s="74"/>
+      <c r="B13" s="71"/>
+      <c r="C13" s="71"/>
       <c r="D13" s="13"/>
       <c r="E13" s="13"/>
       <c r="F13" s="13"/>
@@ -10859,13 +11095,13 @@
       <c r="K13" s="13"/>
     </row>
     <row r="14" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="30" t="s">
+      <c r="B14" s="29" t="s">
         <v>83</v>
       </c>
-      <c r="C14" s="30" t="s">
+      <c r="C14" s="29" t="s">
         <v>72</v>
       </c>
       <c r="D14" s="13"/>
@@ -10891,11 +11127,11 @@
       <c r="K15" s="13"/>
     </row>
     <row r="16" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A16" s="75" t="s">
+      <c r="A16" s="72" t="s">
         <v>63</v>
       </c>
-      <c r="B16" s="76"/>
-      <c r="C16" s="77"/>
+      <c r="B16" s="73"/>
+      <c r="C16" s="74"/>
       <c r="D16" s="13"/>
       <c r="E16" s="13"/>
       <c r="F16" s="13"/>
@@ -10906,13 +11142,13 @@
       <c r="K16" s="12"/>
     </row>
     <row r="17" spans="1:11" ht="15.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A17" s="30" t="s">
+      <c r="A17" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="30" t="s">
+      <c r="B17" s="29" t="s">
         <v>73</v>
       </c>
-      <c r="C17" s="30" t="s">
+      <c r="C17" s="29" t="s">
         <v>74</v>
       </c>
       <c r="D17" s="13"/>
@@ -11105,36 +11341,36 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="79" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="82"/>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
+      <c r="D1" s="79"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A2" s="27" t="s">
+      <c r="A2" s="26" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="27" t="s">
-        <v>106</v>
-      </c>
-      <c r="C2" s="27" t="s">
-        <v>107</v>
-      </c>
-      <c r="D2" s="27" t="s">
-        <v>108</v>
+      <c r="B2" s="26" t="s">
+        <v>100</v>
+      </c>
+      <c r="C2" s="26" t="s">
+        <v>101</v>
+      </c>
+      <c r="D2" s="26" t="s">
+        <v>102</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A3" s="29" t="s">
-        <v>115</v>
-      </c>
-      <c r="B3" s="79" t="s">
+      <c r="A3" s="28" t="s">
         <v>109</v>
       </c>
-      <c r="C3" s="80"/>
-      <c r="D3" s="81"/>
+      <c r="B3" s="76" t="s">
+        <v>103</v>
+      </c>
+      <c r="C3" s="77"/>
+      <c r="D3" s="78"/>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" s="19"/>
@@ -11143,22 +11379,22 @@
       <c r="D4" s="19"/>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A5" s="78" t="s">
-        <v>110</v>
-      </c>
-      <c r="B5" s="78"/>
-      <c r="C5" s="78"/>
+      <c r="A5" s="75" t="s">
+        <v>104</v>
+      </c>
+      <c r="B5" s="75"/>
+      <c r="C5" s="75"/>
       <c r="D5" s="19"/>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A6" s="28" t="s">
+      <c r="A6" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="B6" s="28" t="s">
-        <v>111</v>
-      </c>
-      <c r="C6" s="28" t="s">
-        <v>112</v>
+      <c r="B6" s="27" t="s">
+        <v>105</v>
+      </c>
+      <c r="C6" s="27" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
@@ -11168,22 +11404,22 @@
       <c r="D7" s="19"/>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A8" s="83" t="s">
-        <v>116</v>
-      </c>
-      <c r="B8" s="83"/>
-      <c r="C8" s="83"/>
+      <c r="A8" s="80" t="s">
+        <v>110</v>
+      </c>
+      <c r="B8" s="80"/>
+      <c r="C8" s="80"/>
       <c r="D8" s="19"/>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A9" s="28" t="s">
+      <c r="A9" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="B9" s="28" t="s">
-        <v>113</v>
-      </c>
-      <c r="C9" s="28" t="s">
-        <v>114</v>
+      <c r="B9" s="27" t="s">
+        <v>107</v>
+      </c>
+      <c r="C9" s="27" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
@@ -11199,190 +11435,217 @@
 
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{8C9F8E0C-A578-41B5-B6F5-78192BA475F9}">
-  <dimension ref="A1:E17"/>
+  <dimension ref="A1:F17"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="7" style="19" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="31.140625" style="19" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="14.7109375" style="19" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.85546875" style="19" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="48.140625" style="19" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="19"/>
+    <col min="1" max="1" width="16.42578125" style="110" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="22.5703125" style="110" customWidth="1"/>
+    <col min="3" max="3" width="14.7109375" style="110" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.85546875" style="110" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="26.140625" style="110" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" style="110" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="9.140625" style="110"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="82" t="s">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A1" s="108" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="82"/>
-      <c r="C1" s="82"/>
-      <c r="D1" s="82"/>
-      <c r="E1" s="82"/>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A2" s="27" t="s">
+      <c r="B1" s="108"/>
+      <c r="C1" s="108"/>
+      <c r="D1" s="108"/>
+      <c r="E1" s="109"/>
+      <c r="F1" s="109"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A2" s="111" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="27" t="s">
+      <c r="B2" s="111" t="s">
         <v>86</v>
       </c>
-      <c r="C2" s="27" t="s">
+      <c r="C2" s="111" t="s">
         <v>87</v>
       </c>
-      <c r="D2" s="27" t="s">
+      <c r="D2" s="111" t="s">
         <v>88</v>
       </c>
-      <c r="E2" s="21" t="s">
+      <c r="E2" s="112" t="s">
+        <v>195</v>
+      </c>
+      <c r="F2" s="112"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="113" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="113" t="s">
         <v>89</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="29" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="83" t="s">
+      <c r="C3" s="113"/>
+      <c r="D3" s="113"/>
+      <c r="E3" s="114"/>
+      <c r="F3" s="114"/>
+    </row>
+    <row r="4" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A4" s="115" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="115" t="s">
         <v>90</v>
       </c>
-      <c r="C3" s="83"/>
-      <c r="D3" s="83"/>
-      <c r="E3" s="83"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="31" t="s">
-        <v>58</v>
-      </c>
-      <c r="B4" s="85" t="s">
+      <c r="C4" s="115"/>
+      <c r="D4" s="115"/>
+      <c r="E4" s="116"/>
+      <c r="F4" s="116"/>
+    </row>
+    <row r="5" spans="1:6" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A5" s="117" t="s">
+        <v>76</v>
+      </c>
+      <c r="B5" s="117" t="s">
+        <v>77</v>
+      </c>
+      <c r="C5" s="117"/>
+      <c r="D5" s="117"/>
+      <c r="E5" s="118"/>
+      <c r="F5" s="118"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E6" s="119"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A7" s="120" t="s">
         <v>91</v>
       </c>
-      <c r="C4" s="85"/>
-      <c r="D4" s="85"/>
-      <c r="E4" s="85"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="32" t="s">
-        <v>76</v>
-      </c>
-      <c r="B5" s="84" t="s">
-        <v>77</v>
-      </c>
-      <c r="C5" s="84"/>
-      <c r="D5" s="84"/>
-      <c r="E5" s="84"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="E6" s="8"/>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A7" s="78" t="s">
+      <c r="B7" s="120"/>
+      <c r="C7" s="120"/>
+      <c r="D7" s="120"/>
+      <c r="E7" s="120"/>
+      <c r="F7" s="120"/>
+    </row>
+    <row r="8" spans="1:6" ht="38.25" x14ac:dyDescent="0.2">
+      <c r="A8" s="121" t="s">
+        <v>66</v>
+      </c>
+      <c r="B8" s="121" t="s">
         <v>92</v>
       </c>
-      <c r="B7" s="78"/>
-      <c r="C7" s="78"/>
-      <c r="D7" s="78"/>
-      <c r="E7" s="78"/>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="28" t="s">
+      <c r="C8" s="121" t="s">
+        <v>93</v>
+      </c>
+      <c r="D8" s="121" t="s">
+        <v>196</v>
+      </c>
+      <c r="E8" s="121" t="s">
+        <v>198</v>
+      </c>
+      <c r="F8" s="121" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="E9" s="119"/>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A10" s="114" t="s">
+        <v>94</v>
+      </c>
+      <c r="B10" s="114"/>
+      <c r="C10" s="114"/>
+      <c r="D10" s="114"/>
+      <c r="E10" s="114"/>
+      <c r="F10" s="122"/>
+    </row>
+    <row r="11" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A11" s="123" t="s">
         <v>66</v>
       </c>
-      <c r="B8" s="28" t="s">
+      <c r="B11" s="123" t="s">
+        <v>92</v>
+      </c>
+      <c r="C11" s="123" t="s">
+        <v>95</v>
+      </c>
+      <c r="D11" s="123"/>
+      <c r="E11" s="123" t="s">
+        <v>199</v>
+      </c>
+      <c r="F11" s="121" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A13" s="116" t="s">
+        <v>96</v>
+      </c>
+      <c r="B13" s="116"/>
+      <c r="C13" s="116"/>
+      <c r="D13" s="116"/>
+      <c r="E13" s="116"/>
+      <c r="F13" s="124"/>
+    </row>
+    <row r="14" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A14" s="123" t="s">
+        <v>66</v>
+      </c>
+      <c r="B14" s="123" t="s">
+        <v>92</v>
+      </c>
+      <c r="C14" s="123" t="s">
         <v>93</v>
       </c>
-      <c r="C8" s="28" t="s">
-        <v>94</v>
-      </c>
-      <c r="D8" s="28" t="s">
-        <v>95</v>
-      </c>
-      <c r="E8" s="28" t="s">
-        <v>96</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="E9" s="8"/>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A10" s="83" t="s">
+      <c r="D14" s="123" t="s">
         <v>97</v>
       </c>
-      <c r="B10" s="83"/>
-      <c r="C10" s="83"/>
-      <c r="D10" s="83"/>
-      <c r="E10" s="83"/>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="28" t="s">
+      <c r="E14" s="123" t="s">
+        <v>200</v>
+      </c>
+      <c r="F14" s="121" t="s">
+        <v>197</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A16" s="118" t="s">
+        <v>98</v>
+      </c>
+      <c r="B16" s="118"/>
+      <c r="C16" s="118"/>
+      <c r="D16" s="118"/>
+      <c r="E16" s="118"/>
+      <c r="F16" s="125"/>
+    </row>
+    <row r="17" spans="1:6" ht="25.5" x14ac:dyDescent="0.2">
+      <c r="A17" s="123" t="s">
         <v>66</v>
       </c>
-      <c r="B11" s="28" t="s">
+      <c r="B17" s="123" t="s">
+        <v>92</v>
+      </c>
+      <c r="C17" s="123" t="s">
         <v>93</v>
       </c>
-      <c r="C11" s="28" t="s">
-        <v>98</v>
-      </c>
-      <c r="D11" s="28"/>
-      <c r="E11" s="28" t="s">
+      <c r="D17" s="123" t="s">
         <v>99</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A13" s="85" t="s">
-        <v>100</v>
-      </c>
-      <c r="B13" s="85"/>
-      <c r="C13" s="85"/>
-      <c r="D13" s="85"/>
-      <c r="E13" s="85"/>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="28" t="s">
-        <v>66</v>
-      </c>
-      <c r="B14" s="28" t="s">
-        <v>93</v>
-      </c>
-      <c r="C14" s="28" t="s">
-        <v>94</v>
-      </c>
-      <c r="D14" s="28" t="s">
-        <v>101</v>
-      </c>
-      <c r="E14" s="28" t="s">
-        <v>102</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A16" s="84" t="s">
-        <v>103</v>
-      </c>
-      <c r="B16" s="84"/>
-      <c r="C16" s="84"/>
-      <c r="D16" s="84"/>
-      <c r="E16" s="84"/>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="28" t="s">
-        <v>66</v>
-      </c>
-      <c r="B17" s="28" t="s">
-        <v>104</v>
-      </c>
-      <c r="C17" s="28"/>
-      <c r="D17" s="28"/>
-      <c r="E17" s="28" t="s">
-        <v>105</v>
+      <c r="E17" s="123" t="s">
+        <v>201</v>
+      </c>
+      <c r="F17" s="121" t="s">
+        <v>197</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="8">
-    <mergeCell ref="A1:E1"/>
-    <mergeCell ref="B3:E3"/>
-    <mergeCell ref="B4:E4"/>
-    <mergeCell ref="B5:E5"/>
-    <mergeCell ref="A7:E7"/>
-    <mergeCell ref="A10:E10"/>
-    <mergeCell ref="A13:E13"/>
-    <mergeCell ref="A16:E16"/>
+  <mergeCells count="9">
+    <mergeCell ref="A7:F7"/>
+    <mergeCell ref="A16:F16"/>
+    <mergeCell ref="A13:F13"/>
+    <mergeCell ref="A10:F10"/>
+    <mergeCell ref="E5:F5"/>
+    <mergeCell ref="E4:F4"/>
+    <mergeCell ref="E3:F3"/>
+    <mergeCell ref="E2:F2"/>
+    <mergeCell ref="E1:F1"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="261" orientation="portrait" r:id="rId1"/>
@@ -11394,84 +11657,84 @@
   <dimension ref="A1:E21"/>
   <sheetFormatPr defaultRowHeight="12.75" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="13.5703125" style="24" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="47" style="24" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.28515625" style="24" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="45.28515625" style="24" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="41" style="24" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="9.140625" style="24"/>
+    <col min="1" max="1" width="13.5703125" style="23" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="47" style="23" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.28515625" style="23" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="45.28515625" style="23" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="41" style="23" bestFit="1" customWidth="1"/>
+    <col min="6" max="16384" width="9.140625" style="23"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A1" s="91" t="s">
+      <c r="A1" s="81" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="92"/>
-      <c r="C1" s="92"/>
-      <c r="D1" s="93"/>
+      <c r="B1" s="82"/>
+      <c r="C1" s="82"/>
+      <c r="D1" s="83"/>
       <c r="E1" s="13"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A2" s="20" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="B2" s="20" t="s">
-        <v>118</v>
+        <v>112</v>
       </c>
       <c r="C2" s="20"/>
       <c r="D2" s="20"/>
       <c r="E2" s="12"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A3" s="22" t="s">
+      <c r="A3" s="21" t="s">
+        <v>113</v>
+      </c>
+      <c r="B3" s="21" t="s">
+        <v>114</v>
+      </c>
+      <c r="C3" s="21" t="s">
+        <v>115</v>
+      </c>
+      <c r="D3" s="21"/>
+      <c r="E3" s="13"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A4" s="22" t="s">
+        <v>45</v>
+      </c>
+      <c r="B4" s="36"/>
+      <c r="C4" s="22" t="s">
+        <v>116</v>
+      </c>
+      <c r="D4" s="22" t="s">
+        <v>117</v>
+      </c>
+      <c r="E4" s="13"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A5" s="37" t="s">
+        <v>118</v>
+      </c>
+      <c r="B5" s="37" t="s">
         <v>119</v>
       </c>
-      <c r="B3" s="22" t="s">
+      <c r="C5" s="37" t="s">
+        <v>122</v>
+      </c>
+      <c r="D5" s="25"/>
+      <c r="E5" s="13"/>
+    </row>
+    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
+      <c r="A6" s="38" t="s">
+        <v>58</v>
+      </c>
+      <c r="B6" s="38" t="s">
         <v>120</v>
       </c>
-      <c r="C3" s="22" t="s">
+      <c r="C6" s="38" t="s">
         <v>121</v>
       </c>
-      <c r="D3" s="22"/>
-      <c r="E3" s="13"/>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A4" s="23" t="s">
-        <v>45</v>
-      </c>
-      <c r="B4" s="38"/>
-      <c r="C4" s="23" t="s">
-        <v>122</v>
-      </c>
-      <c r="D4" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="E4" s="13"/>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A5" s="39" t="s">
-        <v>124</v>
-      </c>
-      <c r="B5" s="39" t="s">
-        <v>125</v>
-      </c>
-      <c r="C5" s="39" t="s">
-        <v>128</v>
-      </c>
-      <c r="D5" s="26"/>
-      <c r="E5" s="13"/>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A6" s="40" t="s">
-        <v>58</v>
-      </c>
-      <c r="B6" s="40" t="s">
-        <v>126</v>
-      </c>
-      <c r="C6" s="40" t="s">
-        <v>127</v>
-      </c>
-      <c r="D6" s="41"/>
+      <c r="D6" s="39"/>
       <c r="E6" s="13"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.2">
@@ -11482,26 +11745,26 @@
       <c r="E7" s="12"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A8" s="90" t="s">
-        <v>129</v>
-      </c>
-      <c r="B8" s="90"/>
-      <c r="C8" s="90"/>
-      <c r="D8" s="90"/>
+      <c r="A8" s="88" t="s">
+        <v>123</v>
+      </c>
+      <c r="B8" s="88"/>
+      <c r="C8" s="88"/>
+      <c r="D8" s="88"/>
       <c r="E8" s="13"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A9" s="30" t="s">
+      <c r="A9" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B9" s="42" t="s">
-        <v>132</v>
-      </c>
-      <c r="C9" s="42" t="s">
-        <v>133</v>
-      </c>
-      <c r="D9" s="42" t="s">
-        <v>130</v>
+      <c r="B9" s="40" t="s">
+        <v>126</v>
+      </c>
+      <c r="C9" s="40" t="s">
+        <v>127</v>
+      </c>
+      <c r="D9" s="40" t="s">
+        <v>124</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.2">
@@ -11512,26 +11775,26 @@
       <c r="E10" s="12"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A11" s="89" t="s">
-        <v>131</v>
-      </c>
-      <c r="B11" s="89"/>
-      <c r="C11" s="89"/>
-      <c r="D11" s="89"/>
+      <c r="A11" s="87" t="s">
+        <v>125</v>
+      </c>
+      <c r="B11" s="87"/>
+      <c r="C11" s="87"/>
+      <c r="D11" s="87"/>
       <c r="E11" s="13"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A12" s="30" t="s">
+      <c r="A12" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B12" s="42" t="s">
-        <v>134</v>
-      </c>
-      <c r="C12" s="42" t="s">
-        <v>135</v>
-      </c>
-      <c r="D12" s="42" t="s">
-        <v>136</v>
+      <c r="B12" s="40" t="s">
+        <v>128</v>
+      </c>
+      <c r="C12" s="40" t="s">
+        <v>129</v>
+      </c>
+      <c r="D12" s="40" t="s">
+        <v>130</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.2">
@@ -11542,24 +11805,24 @@
       <c r="E13" s="13"/>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A14" s="88" t="s">
-        <v>137</v>
-      </c>
-      <c r="B14" s="88"/>
-      <c r="C14" s="88"/>
-      <c r="D14" s="88"/>
+      <c r="A14" s="86" t="s">
+        <v>131</v>
+      </c>
+      <c r="B14" s="86"/>
+      <c r="C14" s="86"/>
+      <c r="D14" s="86"/>
       <c r="E14" s="13"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A15" s="30" t="s">
+      <c r="A15" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B15" s="42" t="s">
-        <v>138</v>
-      </c>
-      <c r="C15" s="30"/>
-      <c r="D15" s="42" t="s">
-        <v>139</v>
+      <c r="B15" s="40" t="s">
+        <v>132</v>
+      </c>
+      <c r="C15" s="29"/>
+      <c r="D15" s="40" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.2">
@@ -11570,42 +11833,42 @@
       <c r="E16" s="13"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="87" t="s">
-        <v>140</v>
-      </c>
-      <c r="B17" s="87"/>
-      <c r="C17" s="87"/>
-      <c r="D17" s="87"/>
+      <c r="A17" s="85" t="s">
+        <v>134</v>
+      </c>
+      <c r="B17" s="85"/>
+      <c r="C17" s="85"/>
+      <c r="D17" s="85"/>
       <c r="E17" s="13"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="30" t="s">
+      <c r="A18" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B18" s="42" t="s">
-        <v>141</v>
-      </c>
-      <c r="C18" s="30"/>
-      <c r="D18" s="42" t="s">
-        <v>142</v>
+      <c r="B18" s="40" t="s">
+        <v>135</v>
+      </c>
+      <c r="C18" s="29"/>
+      <c r="D18" s="40" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="86" t="s">
-        <v>143</v>
-      </c>
-      <c r="B20" s="86"/>
-      <c r="C20" s="86"/>
-      <c r="D20" s="86"/>
+      <c r="A20" s="84" t="s">
+        <v>137</v>
+      </c>
+      <c r="B20" s="84"/>
+      <c r="C20" s="84"/>
+      <c r="D20" s="84"/>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A21" s="30" t="s">
+      <c r="A21" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B21" s="42"/>
-      <c r="C21" s="30"/>
-      <c r="D21" s="42" t="s">
-        <v>144</v>
+      <c r="B21" s="40"/>
+      <c r="C21" s="29"/>
+      <c r="D21" s="40" t="s">
+        <v>138</v>
       </c>
     </row>
   </sheetData>
@@ -11635,57 +11898,57 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="79" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="82"/>
-      <c r="C1" s="82"/>
+      <c r="B1" s="79"/>
+      <c r="C1" s="79"/>
       <c r="D1" s="19"/>
       <c r="E1" s="19"/>
       <c r="F1" s="19"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="34" t="s">
+      <c r="A2" s="32" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="34" t="s">
+      <c r="B2" s="32" t="s">
+        <v>139</v>
+      </c>
+      <c r="C2" s="32" t="s">
+        <v>140</v>
+      </c>
+      <c r="D2" s="48"/>
+      <c r="E2" s="48"/>
+      <c r="F2" s="48"/>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="34" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="34" t="s">
+        <v>141</v>
+      </c>
+      <c r="C3" s="34" t="s">
+        <v>142</v>
+      </c>
+      <c r="D3" s="13"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="35" t="s">
+        <v>143</v>
+      </c>
+      <c r="B4" s="49" t="s">
+        <v>144</v>
+      </c>
+      <c r="C4" s="30"/>
+      <c r="D4" s="13"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="31" t="s">
         <v>145</v>
       </c>
-      <c r="C2" s="34" t="s">
-        <v>146</v>
-      </c>
-      <c r="D2" s="51"/>
-      <c r="E2" s="51"/>
-      <c r="F2" s="51"/>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="36" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="36" t="s">
-        <v>147</v>
-      </c>
-      <c r="C3" s="36" t="s">
-        <v>148</v>
-      </c>
-      <c r="D3" s="13"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="37" t="s">
-        <v>149</v>
-      </c>
-      <c r="B4" s="52" t="s">
-        <v>150</v>
-      </c>
-      <c r="C4" s="31"/>
-      <c r="D4" s="13"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="33" t="s">
-        <v>151</v>
-      </c>
-      <c r="B5" s="33"/>
-      <c r="C5" s="33"/>
+      <c r="B5" s="31"/>
+      <c r="C5" s="31"/>
       <c r="D5" s="13"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
@@ -11695,22 +11958,22 @@
       <c r="D6" s="13"/>
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A7" s="98" t="s">
-        <v>152</v>
-      </c>
-      <c r="B7" s="98"/>
-      <c r="C7" s="53"/>
-      <c r="D7" s="53"/>
+      <c r="A7" s="89" t="s">
+        <v>146</v>
+      </c>
+      <c r="B7" s="89"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="50"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="30" t="s">
+      <c r="A8" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B8" s="42" t="s">
-        <v>153</v>
-      </c>
-      <c r="C8" s="51"/>
-      <c r="D8" s="51"/>
+      <c r="B8" s="40" t="s">
+        <v>147</v>
+      </c>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="13"/>
@@ -11719,23 +11982,23 @@
       <c r="D9" s="13"/>
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A10" s="94" t="s">
-        <v>154</v>
-      </c>
-      <c r="B10" s="94"/>
-      <c r="C10" s="53"/>
-      <c r="D10" s="53"/>
-      <c r="E10" s="53"/>
+      <c r="A10" s="90" t="s">
+        <v>148</v>
+      </c>
+      <c r="B10" s="90"/>
+      <c r="C10" s="50"/>
+      <c r="D10" s="50"/>
+      <c r="E10" s="50"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B11" s="42" t="s">
-        <v>155</v>
-      </c>
-      <c r="C11" s="51"/>
-      <c r="D11" s="51"/>
+      <c r="B11" s="40" t="s">
+        <v>149</v>
+      </c>
+      <c r="C11" s="48"/>
+      <c r="D11" s="48"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="13"/>
@@ -11744,23 +12007,23 @@
       <c r="D12" s="13"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="99" t="s">
-        <v>156</v>
-      </c>
-      <c r="B13" s="99"/>
-      <c r="C13" s="53"/>
-      <c r="D13" s="53"/>
-      <c r="E13" s="53"/>
+      <c r="A13" s="91" t="s">
+        <v>150</v>
+      </c>
+      <c r="B13" s="91"/>
+      <c r="C13" s="50"/>
+      <c r="D13" s="50"/>
+      <c r="E13" s="50"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="47" t="s">
-        <v>157</v>
+      <c r="B14" s="45" t="s">
+        <v>151</v>
       </c>
       <c r="C14" s="13"/>
-      <c r="D14" s="51"/>
+      <c r="D14" s="48"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="13"/>
@@ -11769,36 +12032,36 @@
       <c r="D15" s="13"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="95" t="s">
-        <v>158</v>
-      </c>
-      <c r="B16" s="95"/>
-      <c r="C16" s="53"/>
-      <c r="D16" s="53"/>
-      <c r="E16" s="53"/>
+      <c r="A16" s="92" t="s">
+        <v>152</v>
+      </c>
+      <c r="B16" s="92"/>
+      <c r="C16" s="50"/>
+      <c r="D16" s="50"/>
+      <c r="E16" s="50"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="47" t="s">
-        <v>159</v>
+      <c r="B17" s="45" t="s">
+        <v>153</v>
       </c>
       <c r="C17" s="19"/>
-      <c r="D17" s="53"/>
+      <c r="D17" s="50"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="24"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
+      <c r="A18" s="23"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
       <c r="A19" s="13"/>
-      <c r="B19" s="51"/>
-      <c r="C19" s="51"/>
-      <c r="D19" s="51"/>
-      <c r="E19" s="51"/>
+      <c r="B19" s="48"/>
+      <c r="C19" s="48"/>
+      <c r="D19" s="48"/>
+      <c r="E19" s="48"/>
     </row>
   </sheetData>
   <mergeCells count="5">
@@ -11826,56 +12089,56 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A1" s="100" t="s">
+      <c r="A1" s="93" t="s">
         <v>41</v>
       </c>
-      <c r="B1" s="101"/>
-      <c r="C1" s="101"/>
-      <c r="D1" s="102"/>
+      <c r="B1" s="94"/>
+      <c r="C1" s="94"/>
+      <c r="D1" s="95"/>
     </row>
     <row r="2" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A2" s="45" t="s">
+      <c r="A2" s="43" t="s">
         <v>42</v>
       </c>
-      <c r="B2" s="45" t="s">
+      <c r="B2" s="43" t="s">
+        <v>154</v>
+      </c>
+      <c r="C2" s="43" t="s">
+        <v>155</v>
+      </c>
+      <c r="D2" s="43" t="s">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A3" s="42" t="s">
+        <v>45</v>
+      </c>
+      <c r="B3" s="42" t="s">
+        <v>157</v>
+      </c>
+      <c r="C3" s="21"/>
+      <c r="D3" s="21"/>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A4" s="41" t="s">
+        <v>58</v>
+      </c>
+      <c r="B4" s="44" t="s">
+        <v>158</v>
+      </c>
+      <c r="C4" s="22"/>
+      <c r="D4" s="22"/>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+      <c r="A5" s="37" t="s">
+        <v>159</v>
+      </c>
+      <c r="B5" s="37" t="s">
         <v>160</v>
       </c>
-      <c r="C2" s="45" t="s">
-        <v>161</v>
-      </c>
-      <c r="D2" s="45" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A3" s="44" t="s">
-        <v>45</v>
-      </c>
-      <c r="B3" s="44" t="s">
-        <v>163</v>
-      </c>
-      <c r="C3" s="22"/>
-      <c r="D3" s="22"/>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A4" s="43" t="s">
-        <v>58</v>
-      </c>
-      <c r="B4" s="46" t="s">
-        <v>164</v>
-      </c>
-      <c r="C4" s="23"/>
-      <c r="D4" s="23"/>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A5" s="39" t="s">
-        <v>165</v>
-      </c>
-      <c r="B5" s="39" t="s">
-        <v>166</v>
-      </c>
-      <c r="C5" s="39"/>
-      <c r="D5" s="26"/>
+      <c r="C5" s="37"/>
+      <c r="D5" s="25"/>
     </row>
     <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="13"/>
@@ -11885,21 +12148,21 @@
     </row>
     <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="96" t="s">
-        <v>167</v>
+        <v>161</v>
       </c>
       <c r="B7" s="97"/>
-      <c r="C7" s="53"/>
-      <c r="D7" s="53"/>
+      <c r="C7" s="50"/>
+      <c r="D7" s="50"/>
     </row>
     <row r="8" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A8" s="30" t="s">
+      <c r="A8" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B8" s="42" t="s">
-        <v>168</v>
-      </c>
-      <c r="C8" s="51"/>
-      <c r="D8" s="51"/>
+      <c r="B8" s="40" t="s">
+        <v>162</v>
+      </c>
+      <c r="C8" s="48"/>
+      <c r="D8" s="48"/>
     </row>
     <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="13"/>
@@ -11911,23 +12174,23 @@
     </row>
     <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="96" t="s">
-        <v>169</v>
+        <v>163</v>
       </c>
       <c r="B10" s="97"/>
-      <c r="C10" s="53"/>
-      <c r="D10" s="53"/>
-      <c r="E10" s="51"/>
-      <c r="F10" s="51"/>
+      <c r="C10" s="50"/>
+      <c r="D10" s="50"/>
+      <c r="E10" s="48"/>
+      <c r="F10" s="48"/>
     </row>
     <row r="11" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A11" s="30" t="s">
+      <c r="A11" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B11" s="42" t="s">
-        <v>170</v>
-      </c>
-      <c r="C11" s="51"/>
-      <c r="D11" s="51"/>
+      <c r="B11" s="40" t="s">
+        <v>164</v>
+      </c>
+      <c r="C11" s="48"/>
+      <c r="D11" s="48"/>
     </row>
     <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="13"/>
@@ -11936,24 +12199,24 @@
       <c r="D12" s="13"/>
     </row>
     <row r="13" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A13" s="103" t="s">
-        <v>171</v>
-      </c>
-      <c r="B13" s="104"/>
-      <c r="C13" s="53"/>
-      <c r="D13" s="53"/>
+      <c r="A13" s="98" t="s">
+        <v>165</v>
+      </c>
+      <c r="B13" s="99"/>
+      <c r="C13" s="50"/>
+      <c r="D13" s="50"/>
     </row>
     <row r="14" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A14" s="30" t="s">
+      <c r="A14" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B14" s="47" t="s">
-        <v>172</v>
+      <c r="B14" s="45" t="s">
+        <v>166</v>
       </c>
       <c r="C14" s="13"/>
-      <c r="D14" s="51"/>
-      <c r="E14" s="53"/>
-      <c r="F14" s="53"/>
+      <c r="D14" s="48"/>
+      <c r="E14" s="50"/>
+      <c r="F14" s="50"/>
     </row>
     <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="13"/>
@@ -11962,68 +12225,68 @@
       <c r="D15" s="13"/>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.2">
-      <c r="A16" s="99" t="s">
-        <v>173</v>
-      </c>
-      <c r="B16" s="99"/>
-      <c r="C16" s="53"/>
-      <c r="D16" s="53"/>
+      <c r="A16" s="91" t="s">
+        <v>167</v>
+      </c>
+      <c r="B16" s="91"/>
+      <c r="C16" s="50"/>
+      <c r="D16" s="50"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A17" s="28" t="s">
+      <c r="A17" s="27" t="s">
         <v>66</v>
       </c>
-      <c r="B17" s="47" t="s">
-        <v>174</v>
+      <c r="B17" s="45" t="s">
+        <v>168</v>
       </c>
       <c r="C17" s="19"/>
-      <c r="D17" s="53"/>
+      <c r="D17" s="50"/>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A18" s="24"/>
-      <c r="B18" s="24"/>
-      <c r="C18" s="24"/>
-      <c r="D18" s="24"/>
+      <c r="A18" s="23"/>
+      <c r="B18" s="23"/>
+      <c r="C18" s="23"/>
+      <c r="D18" s="23"/>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A19" s="95" t="s">
-        <v>175</v>
-      </c>
-      <c r="B19" s="95"/>
-      <c r="C19" s="53"/>
-      <c r="D19" s="53"/>
-      <c r="E19" s="53"/>
+      <c r="A19" s="92" t="s">
+        <v>169</v>
+      </c>
+      <c r="B19" s="92"/>
+      <c r="C19" s="50"/>
+      <c r="D19" s="50"/>
+      <c r="E19" s="50"/>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A20" s="30" t="s">
+      <c r="A20" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B20" s="42" t="s">
-        <v>176</v>
-      </c>
-      <c r="C20" s="51"/>
-      <c r="D20" s="51"/>
+      <c r="B20" s="40" t="s">
+        <v>170</v>
+      </c>
+      <c r="C20" s="48"/>
+      <c r="D20" s="48"/>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A22" s="95" t="s">
-        <v>177</v>
-      </c>
-      <c r="B22" s="95"/>
-      <c r="E22" s="53"/>
+      <c r="A22" s="92" t="s">
+        <v>171</v>
+      </c>
+      <c r="B22" s="92"/>
+      <c r="E22" s="50"/>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="A23" s="30" t="s">
+      <c r="A23" s="29" t="s">
         <v>66</v>
       </c>
-      <c r="B23" s="42" t="s">
-        <v>178</v>
+      <c r="B23" s="40" t="s">
+        <v>172</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="E25" s="53"/>
+      <c r="E25" s="50"/>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.2">
-      <c r="E28" s="53"/>
+      <c r="E28" s="50"/>
     </row>
   </sheetData>
   <mergeCells count="7">

</xml_diff>